<commit_message>
feat: 2015+ real training, migrate price/yield detail to LGU dashboard, remove farmer price pages, honest metrics with interval
</commit_message>
<xml_diff>
--- a/data/templates/provincial_template.xlsx
+++ b/data/templates/provincial_template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bataan_Dataset" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Palay_Sufficiency_Bataan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Palay_Production_per_Municipali" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bataan_Dataset" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Palay_Sufficiency_Bataan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Palay_Production_per_Municipali" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +27,23 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B5E20"/>
+        <bgColor rgb="001B5E20"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,8 +58,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,88 +431,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Province</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Month_Num</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Production_Irrigated</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Production_Rainfed</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Production_Total</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Production_Annual</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Harvested_Irrigated</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Harvested_Rainfed</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Harvested_Total</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Harvested_Annual</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Fancy_Palay_Price</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Other_Variety_Price</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Quarterly_Yield_MT_per_ha</t>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Production_Irrigated (MT)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Production_Rainfed (MT)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Production_Total (MT)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Production_Annual (MT)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Harvested_Irrigated (ha)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Harvested_Rainfed (ha)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Harvested_Total (ha)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Harvested_Annual (ha)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Fancy_Palay_Price (PHP/kg)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Other_Variety_Price (PHP/kg)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Quarterly_Yield (MT/ha)</t>
         </is>
       </c>
     </row>
@@ -515,29 +531,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Province</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Net Production Clean Rice</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Actual Consumption</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Surplus/Deficit</t>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Net Production Clean Rice (MT)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Actual Consumption (MT)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Surplus/Deficit (MT)</t>
         </is>
       </c>
     </row>
@@ -556,34 +572,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Municipality</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Dry_Season</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Wet_Season</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Palay_Production</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Ave_Production</t>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Dry_Season (MT)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Wet_Season (MT)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Palay_Production (MT)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Ave_Production (MT/ha)</t>
         </is>
       </c>
     </row>

</xml_diff>